<commit_message>
Add new resources and refresh notes in resource database
Adds USFS Geospatial Data Discovery and U.S. Hut Systems, fills in
missing notes, and adds a script to regenerate resources.json from
the dataset_inventory.xlsx spreadsheet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/dataset_inventory.xlsx
+++ b/data/dataset_inventory.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abiga\Portfolio\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AD0ADE9-6D46-46B6-8A97-78BD6984E462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A71C1547-DFA1-4F86-AF2F-26C88B79BC6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-5505" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="149">
   <si>
     <t>Dataset Name</t>
   </si>
@@ -68,9 +68,6 @@
     <t>https://livingatlas.arcgis.com/en/home/</t>
   </si>
   <si>
-    <t>Candid – Search Organizations</t>
-  </si>
-  <si>
     <t>https://candid.org</t>
   </si>
   <si>
@@ -119,9 +116,6 @@
     <t>https://gis-fema.hub.arcgis.com/pages/indices-and-tools</t>
   </si>
   <si>
-    <t>CRAZY amount of information on risk, climate resilience, vulnerability, etc.</t>
-  </si>
-  <si>
     <t>Flood Potential Portal</t>
   </si>
   <si>
@@ -248,9 +242,6 @@
     <t>https://www.usgs.gov/tools/trails-explorer</t>
   </si>
   <si>
-    <t>Wilderness Connect – Wilderness Locator Map</t>
-  </si>
-  <si>
     <t>https://arcg.is/1GCjnS</t>
   </si>
   <si>
@@ -269,12 +260,6 @@
     <t>Maps shelters (with photos), vistas, and other assets along the Appalachian Trail</t>
   </si>
   <si>
-    <t>Super comprehensive collection of different mapping data from around the world</t>
-  </si>
-  <si>
-    <t>Search nonprofits to understand their funding</t>
-  </si>
-  <si>
     <t>Sub-resource of National Equity Atlas that examines car access</t>
   </si>
   <si>
@@ -432,6 +417,69 @@
   </si>
   <si>
     <t>Transportation, Infrastructure</t>
+  </si>
+  <si>
+    <t>Candid</t>
+  </si>
+  <si>
+    <t>Public financial data about non-profits and their funding</t>
+  </si>
+  <si>
+    <t>Huge amount of data on risk, climate resilience, vulnerability, etc.</t>
+  </si>
+  <si>
+    <t>Esri collection of different mapping data from around the world, including maps, apps, and data layers</t>
+  </si>
+  <si>
+    <t>Comprehensive map of all public access lands in the U.S., including privately-held, open access lands, all protected areas, and all managed areas</t>
+  </si>
+  <si>
+    <t>Listing of free-flowing river segments that are believed to possess one or more "outstandingly remarkable" values judged to be of more than local or regional significance</t>
+  </si>
+  <si>
+    <t>Environmental public health data including air quality, built environment, drinking water, disease, etc. and searchable by geography and time</t>
+  </si>
+  <si>
+    <t>Public data on mortalities in national parks</t>
+  </si>
+  <si>
+    <t>Detailed report card on racial and economic equity in the U.S.</t>
+  </si>
+  <si>
+    <t>Authoritative source on the travel behavior of the American public which allows one to analyze trends in personal and household travel</t>
+  </si>
+  <si>
+    <t>USGS aggregated trails viewer</t>
+  </si>
+  <si>
+    <t>Wilderness Locator Map</t>
+  </si>
+  <si>
+    <t>Wilderness Connect map of wilderness locations</t>
+  </si>
+  <si>
+    <t>USFS Geospatial Data Discovery</t>
+  </si>
+  <si>
+    <t>https://data-usfs.hub.arcgis.com/</t>
+  </si>
+  <si>
+    <t>USFS open data site with boundary, asset, and environmental data on national forests</t>
+  </si>
+  <si>
+    <t>Land, Trails, Wilderness, Water</t>
+  </si>
+  <si>
+    <t>U.S. Hut Systems</t>
+  </si>
+  <si>
+    <t>https://www.hutalliance.org/ushutsystems</t>
+  </si>
+  <si>
+    <t>Map of hut systems in the United States</t>
+  </si>
+  <si>
+    <t>Huts, Trails</t>
   </si>
 </sst>
 </file>
@@ -510,7 +558,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -819,7 +867,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
@@ -841,13 +889,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="50" x14ac:dyDescent="0.35">
@@ -858,16 +906,16 @@
         <v>4</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="25" x14ac:dyDescent="0.35">
@@ -878,16 +926,16 @@
         <v>6</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="25" x14ac:dyDescent="0.35">
@@ -898,551 +946,607 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="25" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>78</v>
+        <v>131</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="C6" s="2" t="s">
-        <v>79</v>
+        <v>129</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>15</v>
-      </c>
       <c r="C7" s="2" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="D8" s="2" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>20</v>
-      </c>
       <c r="C9" s="2" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D9" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="F9" s="5" t="s">
         <v>111</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="25" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="D10" s="2" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" s="2"/>
+      <c r="C11" s="2" t="s">
+        <v>134</v>
+      </c>
       <c r="D11" s="2" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="25" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="C12" s="2" t="s">
-        <v>28</v>
+        <v>130</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="E13" s="5" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="D14" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="D15" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="25" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="B16" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
+      <c r="C16" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B17" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="E16" s="5" t="s">
+      <c r="C17" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="25" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E19" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="F16" s="5" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="50" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>114</v>
-      </c>
       <c r="F19" s="5" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B21" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="25" x14ac:dyDescent="0.35">
-      <c r="A21" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C21" s="2"/>
+      <c r="C21" s="2" t="s">
+        <v>133</v>
+      </c>
       <c r="D21" s="2" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="D23" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="B24" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E23" s="5" t="s">
+      <c r="C24" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E24" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="F23" s="5" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="25" x14ac:dyDescent="0.35">
-      <c r="A24" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>109</v>
-      </c>
       <c r="F24" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="25" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>62</v>
-      </c>
       <c r="D26" s="2" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="87.5" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="25" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>68</v>
-      </c>
       <c r="D29" s="2" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="E29" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="25" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B30" t="s">
+        <v>142</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E30" s="5" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A30" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>109</v>
-      </c>
       <c r="F30" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B32" t="s">
+        <v>146</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B34" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="E31" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A32" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="E32" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>81</v>
+      <c r="C34" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1455,7 +1559,14 @@
     <hyperlink ref="B25" r:id="rId6" location="tools" xr:uid="{7E999D70-B411-42FF-8C53-B6AF3A2DBB05}"/>
     <hyperlink ref="B27" r:id="rId7" xr:uid="{D4A02BE3-B4E9-49E3-B661-6228B78A50EC}"/>
     <hyperlink ref="B15" r:id="rId8" xr:uid="{1FE3F742-C541-4274-A45E-D7FADAC9C2A9}"/>
-    <hyperlink ref="B32" r:id="rId9" xr:uid="{B641EC6D-3FAC-481F-9400-7F1B08500579}"/>
+    <hyperlink ref="B34" r:id="rId9" xr:uid="{B641EC6D-3FAC-481F-9400-7F1B08500579}"/>
+    <hyperlink ref="B5" r:id="rId10" xr:uid="{2F9B5A91-8155-4775-B6D0-8EAA1C322185}"/>
+    <hyperlink ref="B24" r:id="rId11" xr:uid="{4310BA34-7474-490D-BCFE-3AA8BBF50ED8}"/>
+    <hyperlink ref="B21" r:id="rId12" xr:uid="{26B7C03D-4125-4EAB-BC47-AE45B91DD380}"/>
+    <hyperlink ref="B17" r:id="rId13" location=":~:text=Key%20Mortality%20Statistics%3A%201%20A%20total%20of%20990,U.S.%20population%20%28844%20deaths%2F100%2C000%20people%29%20%5B2%5D%20More%20items" xr:uid="{7259DF99-FDE1-49C6-B31C-5338FBFE2C4D}"/>
+    <hyperlink ref="B18" r:id="rId14" xr:uid="{B6982ECA-0384-42B6-B05C-A1BA86F56283}"/>
+    <hyperlink ref="B19" r:id="rId15" xr:uid="{D53D3811-295E-4C97-8863-482F44476D90}"/>
+    <hyperlink ref="B31" r:id="rId16" xr:uid="{0FF15D71-9969-4623-BB58-28D73861C428}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>